<commit_message>
Split Nexteer Automotive from HTF ACD Nexteer (C132)
Add C132 Nexteer Automotive India Pvt. Ltd to Customer Master and point
Nexteer OCR aliases to C132 instead of C044 so output folders use the legal
customer name, not HTF ACD Nexteer.

Co-authored-by: ananta126 <ananta126@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/invoice_sorter_app_v2/customer_master_alias_mapping.xlsx
+++ b/invoice_sorter_app_v2/customer_master_alias_mapping.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer Master" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alias Master" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Required" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Matches" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping Audit" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Customer Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Alias Master" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Review Required" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="All Matches" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Mapping Audit" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Customer Master'!$A$1:$B$110</definedName>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B130"/>
+  <dimension ref="A1:B131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2012,6 +2012,18 @@
       <c r="B130" t="inlineStr">
         <is>
           <t>VISHAL ENGINEERS PVT.LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>C132</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Nexteer Automotive India Pvt. Ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert Nexteer aliases to confirmed C044 (HTF ACD Nexteer)
Remove unconfirmed C132 customer row from master xlsx. Regression tests
for EXACT_ALIAS match and COMPLETED sort under HTF ACD Nexteer folder.

Co-authored-by: ananta126 <ananta126@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/invoice_sorter_app_v2/customer_master_alias_mapping.xlsx
+++ b/invoice_sorter_app_v2/customer_master_alias_mapping.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B131"/>
+  <dimension ref="A1:B130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2012,18 +2012,6 @@
       <c r="B130" t="inlineStr">
         <is>
           <t>VISHAL ENGINEERS PVT.LTD</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>C132</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>Nexteer Automotive India Pvt. Ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore C132 Nexteer India split from HTF ACD Nexteer (C044)
Re-add C132 to Customer Master; point Nexteer legal-name OCR aliases to C132.
HTF ACD Nexteer remains C044 via EXACT_OFFICIAL. Tests cover sort routing.

Co-authored-by: ananta126 <ananta126@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/invoice_sorter_app_v2/customer_master_alias_mapping.xlsx
+++ b/invoice_sorter_app_v2/customer_master_alias_mapping.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B130"/>
+  <dimension ref="A1:B131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2012,6 +2012,18 @@
       <c r="B130" t="inlineStr">
         <is>
           <t>VISHAL ENGINEERS PVT.LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>C132</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Nexteer Automotive India Pvt. Ltd</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3592,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>C044</t>
+          <t>C132</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3604,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>C044</t>
+          <t>C132</t>
         </is>
       </c>
     </row>
@@ -3604,7 +3616,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>C044</t>
+          <t>C132</t>
         </is>
       </c>
     </row>
@@ -3616,7 +3628,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>C044</t>
+          <t>C132</t>
         </is>
       </c>
     </row>
@@ -3628,7 +3640,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>C044</t>
+          <t>C132</t>
         </is>
       </c>
     </row>
@@ -3640,7 +3652,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>C044</t>
+          <t>C132</t>
         </is>
       </c>
     </row>

</xml_diff>